<commit_message>
ajout fichier des modifications du fichier connaissances
</commit_message>
<xml_diff>
--- a/Bases de Connaissances.xlsx
+++ b/Bases de Connaissances.xlsx
@@ -1,22 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Invite\Documents\LABsODC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\Documents\projet_portfolio\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F562308B-5362-4647-8E6C-686A82C8F600}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{460EB59E-A833-4371-A464-1FFBE0E81E70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{72921A0A-C693-4A8D-AAD6-8BC21755823B}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{72921A0A-C693-4A8D-AAD6-8BC21755823B}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -26,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="48">
   <si>
     <t>Problème n°</t>
   </si>
@@ -269,12 +268,35 @@
   <si>
     <t>exemple 4</t>
   </si>
+  <si>
+    <t>Ex. 5</t>
+  </si>
+  <si>
+    <t>Services Aws</t>
+  </si>
+  <si>
+    <t>Lors de l'exécution du script create-instance.sh, la création d'une instance EC2 échoue. Le script est censé automatiser le déploiement d'un serveur café (cafeserver) sur AWS EC2 en récupérant dynamiquement les paramètres nécessaires (VPC, Subnet, AMI, Security Group, etc.), mais plusieurs erreurs empêchent son bon fonctionnement.</t>
+  </si>
+  <si>
+    <t>An error occurred (InvalidAMIID.NotFound) when calling the 
+RunInstances operation: The image id '[ami-0794771afcf01a21f]' 
+does not exist</t>
+  </si>
+  <si>
+    <t>la region était diffrente avec celle de l'AMI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Résolution 1 — Fixer la variable région
+La région n'est jamais déclarée explicitement en variable. Résolution 2 — Corriger la récupération de l'AMI ID
+ L'utilisation de grep | cut | sed produit un résultat avec des crochets [ ].Résolution 3 — Corriger la région dans run-instances
+La région est codée en dur à us-east-1 dans la commande run-instances alors que toutes les ressources sont en us-west-2.              </t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -352,6 +374,12 @@
       <color rgb="FF000000"/>
       <name val="Amazon Ember Light"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="6">
@@ -884,18 +912,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{000852F0-EFD2-49C1-9E80-6455AD63EA5E}">
-  <dimension ref="A1:I5"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <dimension ref="A1:I6"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="24.140625" customWidth="1"/>
-    <col min="2" max="2" width="26.7109375" customWidth="1"/>
-    <col min="3" max="3" width="60.42578125" customWidth="1"/>
-    <col min="4" max="4" width="58.42578125" customWidth="1"/>
-    <col min="5" max="5" width="28.140625" customWidth="1"/>
-    <col min="6" max="6" width="95.140625" customWidth="1"/>
-    <col min="7" max="7" width="65.7109375" customWidth="1"/>
-    <col min="8" max="8" width="54.85546875" customWidth="1"/>
-    <col min="9" max="9" width="67.28515625" customWidth="1"/>
+    <col min="1" max="1" width="24.1796875" customWidth="1"/>
+    <col min="2" max="2" width="26.7265625" customWidth="1"/>
+    <col min="3" max="3" width="60.453125" customWidth="1"/>
+    <col min="4" max="4" width="58.453125" customWidth="1"/>
+    <col min="5" max="5" width="28.1796875" customWidth="1"/>
+    <col min="6" max="6" width="95.1796875" customWidth="1"/>
+    <col min="7" max="7" width="65.7265625" customWidth="1"/>
+    <col min="8" max="8" width="54.81640625" customWidth="1"/>
+    <col min="9" max="9" width="67.26953125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" s="4" customFormat="1" ht="77.25" customHeight="1" thickBot="1">
@@ -1041,7 +1069,28 @@
         <v>41</v>
       </c>
     </row>
+    <row r="6" spans="1:9" ht="160.5" thickBot="1">
+      <c r="A6" s="17" t="s">
+        <v>42</v>
+      </c>
+      <c r="B6" s="18" t="s">
+        <v>43</v>
+      </c>
+      <c r="C6" s="19" t="s">
+        <v>44</v>
+      </c>
+      <c r="D6" s="19" t="s">
+        <v>45</v>
+      </c>
+      <c r="E6" s="19" t="s">
+        <v>46</v>
+      </c>
+      <c r="F6" s="19" t="s">
+        <v>47</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="12" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
ajout du fichier de probleme de depannage
</commit_message>
<xml_diff>
--- a/Bases de Connaissances.xlsx
+++ b/Bases de Connaissances.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\Documents\projet_portfolio\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE5111BA-2B13-4780-B49E-400AE73DD8F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91F9844B-AFCB-4E1A-AF3F-EBE1FF39FF22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{72921A0A-C693-4A8D-AAD6-8BC21755823B}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="69">
   <si>
     <t>Problème n°</t>
   </si>
@@ -321,6 +321,45 @@
   </si>
   <si>
     <t xml:space="preserve">on a demarré le service httpd et l'activer </t>
+  </si>
+  <si>
+    <t>Ex. 8</t>
+  </si>
+  <si>
+    <t>Depanner un vpc</t>
+  </si>
+  <si>
+    <t>La cause racine ici est une règle DENY trop large dans l'ACL réseau du sous-réseau public. Contrairement aux groupes de sécurité (qui sont avec état et n'autorisent que ce qui est explicitement permis), les ACL réseau sont sans état et sont évaluées par numéro de règle croissant — la première règle qui correspond est appliquée</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Etablishing connexion ssh  </t>
+  </si>
+  <si>
+    <t>l'acl presentait une regle deny qui empechait la connexion ssh</t>
+  </si>
+  <si>
+    <t>Ex. 9</t>
+  </si>
+  <si>
+    <t>Supprimer la règle DENY problématique
+aws ec2 delete-network-acl-entry --network-acl-id 'acl-xxxxx'
+--rule-number 1 --ingress
+Résultat : trafic SSH (22) et HTTP (80) déblocqués vers l'instance</t>
+  </si>
+  <si>
+    <t>La cause racine la plus probable dans ce scénario est l'absence de la route par défaut (0.0.0.0/0) vers l'Internet Gateway dans la table de routage du sous-réseau public. Sans cette route, les paquets n'ont pas de chemin vers Internet, même si le groupe de sécurité autorise le trafic.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Site web inaccessible </t>
+  </si>
+  <si>
+    <t>l'absence de route  par defaut vers l'internet gateway</t>
+  </si>
+  <si>
+    <t>aws ec2 create-route \
+  --route-table-id 'VPC1PubRouteTableId' \
+  --gateway-id 'VPC1GatewayId' \
+  --destination-cidr-block '0.0.0.0/0'</t>
   </si>
 </sst>
 </file>
@@ -943,7 +982,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{000852F0-EFD2-49C1-9E80-6455AD63EA5E}">
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="24.1796875" customWidth="1"/>
@@ -1133,6 +1172,7 @@
       <c r="D7" s="19" t="s">
         <v>48</v>
       </c>
+      <c r="E7" s="19"/>
       <c r="F7" s="19" t="s">
         <v>50</v>
       </c>
@@ -1150,8 +1190,49 @@
       <c r="D8" s="19" t="s">
         <v>56</v>
       </c>
+      <c r="E8" s="19"/>
       <c r="F8" s="19" t="s">
         <v>57</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="160.5" thickBot="1">
+      <c r="A9" s="17" t="s">
+        <v>58</v>
+      </c>
+      <c r="B9" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="C9" s="19" t="s">
+        <v>60</v>
+      </c>
+      <c r="D9" s="19" t="s">
+        <v>61</v>
+      </c>
+      <c r="E9" s="19" t="s">
+        <v>62</v>
+      </c>
+      <c r="F9" s="19" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="140.5" thickBot="1">
+      <c r="A10" s="17" t="s">
+        <v>63</v>
+      </c>
+      <c r="B10" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="C10" s="19" t="s">
+        <v>65</v>
+      </c>
+      <c r="D10" s="19" t="s">
+        <v>66</v>
+      </c>
+      <c r="E10" s="19" t="s">
+        <v>67</v>
+      </c>
+      <c r="F10" s="19" t="s">
+        <v>68</v>
       </c>
     </row>
   </sheetData>

</xml_diff>